<commit_message>
More updates in preparation for sharing Draft with public
</commit_message>
<xml_diff>
--- a/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist_DRAFT.xlsx
+++ b/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist_DRAFT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flankspeed-my.sharepoint-mil.us/personal/jack_r_vanderpol_civ_us_navy_mil/Documents/Documents/github/SCAP-Self-Assertion/SCAP_1.4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="163" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC1CDAAE-9536-4FC8-BF69-DA072706C2D2}"/>
+  <xr:revisionPtr revIDLastSave="229" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C3F3B37-486F-443F-A6E1-64FE5EFB87ED}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="90" windowWidth="29040" windowHeight="15510" xr2:uid="{91EDF8AA-12A4-463E-9EF6-D256E525D567}"/>
+    <workbookView xWindow="-120" yWindow="90" windowWidth="29040" windowHeight="15510" activeTab="2" xr2:uid="{91EDF8AA-12A4-463E-9EF6-D256E525D567}"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="SCAP 1.4 Self Assertion" sheetId="1" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SCAP 1.4 Self Assertion'!$A$1:$N$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SCAP 1.4 Self Assertion'!$A$1:$N$60</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'SCAP 1.4 Self Assertion'!$A:$J</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="314">
   <si>
     <t>The product’s documentation (printed or electronic) MUST assert that it uses SCAP and its component specifications and explain relevant details to the users of the product.</t>
   </si>
@@ -189,9 +189,6 @@
     <t>SCAP.T.700.1: The tester SHALL validate that the vendor product can selectively choose and apply a specific valid XCCDF profile.</t>
   </si>
   <si>
-    <t>Install SCAP 1.4 content from NIWC repository, view several profiles and perform scans from more than one profile.</t>
-  </si>
-  <si>
     <t>SCAP.R.800</t>
   </si>
   <si>
@@ -203,10 +200,6 @@
 SCAP.T.800.3: The tester SHALL import a valid signed SCAP source data stream into the vendor product and ensure that the imported content is available for execution.</t>
   </si>
   <si>
-    <t>Install unsigned content from DISA's SCAP 1.3 repository.
-Install signed content from NIWC's SCAP 1.4 repository</t>
-  </si>
-  <si>
     <t>SCAP.R.900</t>
   </si>
   <si>
@@ -216,10 +209,6 @@
     <t>SCAP.T.900.1: The tester SHALL verify that the product documentation includes instructions on how the digital signature is validated.
 SCAP.T.900.2: The tester SHALL verify that the vendor product can correctly validate the digital signature of a source data stream.
 SCAP.T.900.3: The tester SHALL verify that the vendor product correctly identifies and reports an error when processing a data stream with an invalid digital signature.</t>
-  </si>
-  <si>
-    <t>Install content that is signed and unmodified, verify that it reports sucessful digital signature validation.
-Install content that is signed, but has been modified, and attempt to perform a scan.  Application should at minimum report an error and may reject running the content, based on optional application configuration settings.</t>
   </si>
   <si>
     <t>SCAP.R.1000</t>
@@ -740,9 +729,6 @@
     <t>Since USGCB is no longer required, this test should be removed, unless we want to state that applications need to be compliant with all DISA STIGs?  Would take some research to know if that is possible or wise.</t>
   </si>
   <si>
-    <t>Removed OVAL Repository note, as it's no longer existent.</t>
-  </si>
-  <si>
     <t>Updated to 800-126 R4</t>
   </si>
   <si>
@@ -821,11 +807,6 @@
     <t>SCAP.V.4100.1: The vendor SHALL supply documentation on how to import an SCAP data stream, apply it against a target, and produce an SCAP result data stream conforming to the ARF specification.</t>
   </si>
   <si>
-    <t>SCAP.T.4100.1: The tester SHALL import the SCAP 1.3 source data stream, apply it to a known target, and produce an SCAP result data stream conforming to the ARF specification.
-SCAP.T.4100.2: The tester SHALL validate the results produced using SCAPVal; the validation MUST NOT produce any errors.
-SCAP.T.4100.3: The tester SHALL compare the actual results to the expected results ensuring the results match.</t>
-  </si>
-  <si>
     <t>SCAP.R.4200</t>
   </si>
   <si>
@@ -940,9 +921,6 @@
     <t>SCAP.V.5008.1:  The vendor SHALL provide documentation listing all supported operating systems.</t>
   </si>
   <si>
-    <t>SCAP.R.5009</t>
-  </si>
-  <si>
     <t>SCAP.V.5009.1:  The vendor SHALL provide documentation listing all supported operating systems.</t>
   </si>
   <si>
@@ -964,13 +942,7 @@
     <t>If the product supports Cisco IOS-XE, it SHALL support OVAL 5.12.2 tests for ios-xe  schemas along with all core OVAL 5.12.2 features.</t>
   </si>
   <si>
-    <t>If the product supports ESX, it SHALL support all non-deprecated OVAL 5.12.2 tests ESX  schemas along with all core OVAL 5.12 features.</t>
-  </si>
-  <si>
     <t>If the product supports AWS, it SHALL support all non-deprecated OVAL 5.12.2 tests AWS  schemas along with all core OVAL 5.12 features.</t>
-  </si>
-  <si>
-    <t>Install SCAP 1.3 content from DISA's repository</t>
   </si>
   <si>
     <t>NIWC Comments</t>
@@ -1030,10 +1002,6 @@
   </si>
   <si>
     <t>SCAP.T.5008.1:  The tester SHALL install the OVAL test content and scan using all PANOS content, along with all agnostic content designed to demonstrate support of OVAL 5.12.2.
-Any non supported tests must be documented.</t>
-  </si>
-  <si>
-    <t>SCAP.T.5009.1:  The tester SHALL install the OVAL test content and scan using all ESX content, along with all agnostic content designed to demonstrate support of OVAL 5.12.2.
 Any non supported tests must be documented.</t>
   </si>
   <si>
@@ -1154,6 +1122,120 @@
     d. Vendor or Application Logo ( 300 x 300 square in PNG Format)
 </t>
     </r>
+  </si>
+  <si>
+    <t>1.  Install and run any single SCAP 1.4 content stream that is supported by the SCAP interpreter under testcase
+2.  Select a profile a perform a scan
+3.  Perform scans, ensuring that XML results are schema valid.
+4.  No errors are reported.</t>
+  </si>
+  <si>
+    <t>1.  Install and run any single SCAP 1.4 content stream from the \SCAP_Test_Content\R1500 directory that is supported by the SCAP interpreter under testcase
+2.  Select a profile a perform a scan
+3.  Perform scans, ensuring that XML results are schema valid.
+4.  No errors are reported.</t>
+  </si>
+  <si>
+    <t>1.  Attempt to install the SCAP 1.4 content in the SCAP_Test_Content\R1400 directory
+2.  XML schema validation errors should be reported, related to OCIL</t>
+  </si>
+  <si>
+    <t>1.  Install U_MS_Defender_Antivirus_V2R7_STIG_SCAP_1-4_Benchmark-enhancedV13-signed.zip
+a.  Content should install and scans posible with a valid XML digital signature
+2.  Install U_MS_Edge_V2R4_STIG_SCAP_1-4_Benchmark-enhancedV14-corrupt.zip
+a.  Scanner should report that the XML digital signature validaton failed, and refuse to perform a scan.</t>
+  </si>
+  <si>
+    <t>SCAP.T.800.2
+1.  Refer to DISA STIG SCAP 1.3 unsigned benchmarks in the R1100 folder
+a.  Install and scan one that is applicable to the system being tested.
+SCAP.T.800.3
+1.  Refer to NIWC STIG SCAP 1.4 signed benchmarks in the R700 folder
+a.  Install and scan one that is applicable to the system being tested.</t>
+  </si>
+  <si>
+    <t>1.  Install and run all content that the SCAP interpreter under test supports
+2.  Perform scans, ensuring that XML results are schema valid.
+3.  No errors are reported.</t>
+  </si>
+  <si>
+    <t>Seems redundant to R700 and R1500, potentially remove?</t>
+  </si>
+  <si>
+    <t>SCAP.T.4100.1: The tester SHALL import the SCAP 1.4 source data stream, apply it to a known target, and produce an SCAP result data stream conforming to the ARF specification.
+SCAP.T.4100.2: The tester SHALL validate the results produced using SCAPVal; the validation MUST NOT produce any errors.
+SCAP.T.4100.3: The tester SHALL compare the actual results to the expected results ensuring the results match.</t>
+  </si>
+  <si>
+    <t>Use SCAP_Test_Content\R2920 test content.</t>
+  </si>
+  <si>
+    <t>Test Benchmark Applicability:
+1. Select one of the content streams in SCAP_Test_Content\R1200 that is not applicable to the target OS
+ex.  Scan Windows with MacOS content or MacOS with Linux etc..
+2. SCAP interpreter should refuse to perform the scan and report that the content is not applicable to the target.
+3. Then select a content stream  from SCAP_Test_Content\R1200 that is applicable to the target system
+ex.  Scan Windows 11 with Windows 11 content etc..
+4. SCAP interpreter should report that the content is applicable and perform the scan.
+Test Rule Applicability:
+- This will require either a Windows Server OS (not configured as a domain controller, or a RHEL/Oracle Linux system configured without a Gnome desktop.
+1.  Review the Windows OS, and review rule results, confirming that domain controller specific rules are reported as not_applicable.
+or
+1.  Review an Oracle or RHEL system and review rule results, confirming that any Gnome specific requirements are reported as not_applicable.</t>
+  </si>
+  <si>
+    <t>Recommend removing requirement.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\agnostic.
+2.  Install all OVAL content from OVAL_Test_Content\windows.
+3.  Scan Windows targets with all OVAL content from steps 1-2, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\agnostic.
+2.  Install all OVAL content from OVAL_Test_Content\linux.
+3.  Install all OVAL content from OVAL_Test_Content\unix.
+4.  Scan Linux targets with all OVAL content from steps 1-3, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\agnostic.
+2.  Install all OVAL content from OVAL_Test_Content\macos.
+3.  Scan macOS targets with all OVAL content from steps 1-2, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\agnostic.
+2.  Install all OVAL content from OVAL_Test_Content\solaris.
+3.  Install all OVAL content from OVAL_Test_Content\unix.
+4.  Scan Solaris targets with all OVAL content from steps 1-3, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\ios.
+2.  Scan cisco targets with all OVAL content from step 1, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\ios-xe.
+2.  Scan cisco-xe targets with all OVAL content from step 1, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\junos.
+2.  Scan junos targets with all OVAL content from step 1, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\aws.
+2.  Scan aws targets with all OVAL content from step 1, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\panos.
+2.  Scan panos targets with all OVAL content from step 1, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
   </si>
 </sst>
 </file>
@@ -1652,12 +1734,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
     </row>
   </sheetData>
@@ -1680,69 +1762,69 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>293</v>
+        <v>284</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="B2" s="7"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="B3" s="7"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="B4" s="7"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="B5" s="7"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="B6" s="7"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="B7" s="7"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="B8" s="7"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="B9" s="7"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="B10" s="7"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="B11" s="7"/>
     </row>
@@ -1757,17 +1839,17 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:W62"/>
+  <dimension ref="A1:W61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" style="18" customWidth="1"/>
-    <col min="2" max="2" width="6.7109375" style="18" customWidth="1"/>
+    <col min="2" max="2" width="6.7109375" style="18" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="7.5703125" style="18" customWidth="1"/>
     <col min="4" max="4" width="14.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="38.42578125" style="3" customWidth="1"/>
     <col min="6" max="6" width="45.140625" style="3" customWidth="1"/>
     <col min="7" max="7" width="49" style="3" customWidth="1"/>
-    <col min="8" max="8" width="31.140625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="37.7109375" style="3" customWidth="1"/>
     <col min="9" max="9" width="22.42578125" style="3" customWidth="1"/>
     <col min="10" max="10" width="11.28515625" style="3" customWidth="1"/>
     <col min="11" max="11" width="13.140625" style="18" customWidth="1"/>
@@ -1786,16 +1868,16 @@
         <v>5</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>21</v>
@@ -1807,19 +1889,19 @@
         <v>9</v>
       </c>
       <c r="K1" s="12" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="M1" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="W1" s="13" t="s">
         <v>268</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>269</v>
-      </c>
-      <c r="W1" s="13" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="105" x14ac:dyDescent="0.25">
@@ -1848,7 +1930,7 @@
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
       <c r="W2" s="3" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="210" x14ac:dyDescent="0.25">
@@ -1856,28 +1938,28 @@
       <c r="B3" s="14"/>
       <c r="C3" s="14"/>
       <c r="D3" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
       <c r="K3" s="14"/>
       <c r="L3" s="2" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="W3" s="3" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="135" x14ac:dyDescent="0.25">
@@ -1893,7 +1975,7 @@
         <v>10</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -1906,7 +1988,7 @@
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
     </row>
-    <row r="5" spans="1:23" ht="225" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" ht="210" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>6</v>
       </c>
@@ -1947,7 +2029,7 @@
         <v>18</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>19</v>
@@ -1962,7 +2044,7 @@
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
     </row>
-    <row r="7" spans="1:23" ht="285" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" ht="225" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>6</v>
       </c>
@@ -1990,7 +2072,7 @@
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
     </row>
-    <row r="8" spans="1:23" ht="75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" ht="105" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>6</v>
       </c>
@@ -2009,7 +2091,7 @@
         <v>32</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>33</v>
+        <v>294</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -2025,19 +2107,19 @@
       <c r="B9" s="14"/>
       <c r="C9" s="14"/>
       <c r="D9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="H9" s="2" t="s">
-        <v>37</v>
+        <v>298</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -2046,26 +2128,26 @@
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
     </row>
-    <row r="10" spans="1:23" ht="195" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" ht="180" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>
       <c r="D10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="H10" s="2" t="s">
-        <v>41</v>
+        <v>297</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -2081,10 +2163,10 @@
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
       <c r="D11" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -2093,65 +2175,67 @@
       <c r="J11" s="2"/>
       <c r="K11" s="14"/>
       <c r="L11" s="2" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
     </row>
-    <row r="12" spans="1:23" ht="60" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
       <c r="D12" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>266</v>
+        <v>299</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="14"/>
       <c r="L12" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
     </row>
-    <row r="13" spans="1:23" ht="195" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B13" s="14"/>
       <c r="C13" s="14"/>
       <c r="D13" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H13" s="2"/>
+        <v>46</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>303</v>
+      </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="14"/>
       <c r="L13" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
@@ -2163,19 +2247,19 @@
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
       <c r="D14" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="H14" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -2191,18 +2275,20 @@
         <v>6</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="H15" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>296</v>
+      </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="14"/>
@@ -2210,23 +2296,25 @@
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
     </row>
-    <row r="16" spans="1:23" ht="105" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" ht="135" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="14"/>
       <c r="D16" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
+      <c r="H16" s="2" t="s">
+        <v>295</v>
+      </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="14"/>
@@ -2241,16 +2329,16 @@
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
       <c r="D17" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G17" s="5" t="s">
         <v>71</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>74</v>
       </c>
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
@@ -2259,31 +2347,33 @@
         <v>6</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
     </row>
     <row r="18" spans="1:14" ht="105" x14ac:dyDescent="0.25">
-      <c r="A18" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>76</v>
+      <c r="A18" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
-      <c r="K18" s="14"/>
+      <c r="K18" s="14" t="s">
+        <v>6</v>
+      </c>
       <c r="L18" s="2" t="s">
-        <v>191</v>
+        <v>300</v>
       </c>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
@@ -2295,16 +2385,16 @@
         <v>6</v>
       </c>
       <c r="D19" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="G19" s="5" t="s">
         <v>77</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>80</v>
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
@@ -2323,16 +2413,16 @@
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
       <c r="D20" s="5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
@@ -2349,25 +2439,27 @@
         <v>6</v>
       </c>
       <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="14"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="14" t="s">
+        <v>6</v>
+      </c>
       <c r="L21" s="2" t="s">
-        <v>192</v>
+        <v>304</v>
       </c>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
@@ -2379,19 +2471,19 @@
         <v>6</v>
       </c>
       <c r="D22" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="H22" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>91</v>
       </c>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
@@ -2407,16 +2499,16 @@
         <v>6</v>
       </c>
       <c r="D23" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
@@ -2433,16 +2525,16 @@
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
       <c r="D24" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G24" s="5" t="s">
         <v>96</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>99</v>
       </c>
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
@@ -2451,7 +2543,7 @@
         <v>6</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
@@ -2463,16 +2555,16 @@
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
       <c r="D25" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="G25" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>103</v>
       </c>
       <c r="H25" s="5"/>
       <c r="I25" s="2"/>
@@ -2481,7 +2573,7 @@
         <v>6</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
@@ -2493,16 +2585,16 @@
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
       <c r="D26" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="G26" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>107</v>
       </c>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
@@ -2511,7 +2603,7 @@
         <v>6</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
@@ -2521,23 +2613,23 @@
       <c r="B27" s="14"/>
       <c r="C27" s="14"/>
       <c r="D27" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="14"/>
       <c r="L27" s="2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
@@ -2545,20 +2637,20 @@
     <row r="28" spans="1:14" ht="285" x14ac:dyDescent="0.25">
       <c r="A28" s="15"/>
       <c r="B28" s="15" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C28" s="15"/>
       <c r="D28" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="G28" s="5" t="s">
         <v>111</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>114</v>
       </c>
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
@@ -2567,7 +2659,7 @@
         <v>6</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="M28" s="1"/>
       <c r="N28" s="1"/>
@@ -2575,20 +2667,20 @@
     <row r="29" spans="1:14" ht="180" x14ac:dyDescent="0.25">
       <c r="A29" s="15"/>
       <c r="B29" s="15" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C29" s="15"/>
       <c r="D29" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="G29" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="H29" s="5"/>
       <c r="I29" s="2"/>
@@ -2597,7 +2689,7 @@
         <v>6</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="M29" s="1"/>
       <c r="N29" s="1"/>
@@ -2609,16 +2701,16 @@
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
       <c r="D30" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="G30" s="5" t="s">
         <v>119</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>122</v>
       </c>
       <c r="H30" s="5"/>
       <c r="I30" s="2"/>
@@ -2627,7 +2719,7 @@
         <v>6</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
@@ -2639,23 +2731,23 @@
       <c r="B31" s="16"/>
       <c r="C31" s="16"/>
       <c r="D31" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31" s="2"/>
       <c r="K31" s="16"/>
       <c r="L31" s="2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
@@ -2667,16 +2759,16 @@
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
       <c r="D32" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="F32" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="E32" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>134</v>
-      </c>
       <c r="G32" s="5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
@@ -2685,7 +2777,7 @@
         <v>6</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
@@ -2697,53 +2789,55 @@
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G33" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="E33" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="H33" s="1"/>
+      <c r="H33" s="1" t="s">
+        <v>302</v>
+      </c>
       <c r="I33" s="1"/>
       <c r="J33" s="2"/>
       <c r="K33" s="16"/>
       <c r="L33" s="2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
     </row>
-    <row r="34" spans="1:14" ht="240" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" ht="195" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B34" s="16"/>
       <c r="C34" s="16"/>
       <c r="D34" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E34" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="G34" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="F34" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>142</v>
-      </c>
       <c r="H34" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="I34" s="1"/>
       <c r="J34" s="2"/>
       <c r="K34" s="16"/>
       <c r="L34" s="2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
@@ -2755,23 +2849,23 @@
       <c r="B35" s="16"/>
       <c r="C35" s="16"/>
       <c r="D35" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="G35" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>146</v>
       </c>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
       <c r="J35" s="2"/>
       <c r="K35" s="16"/>
       <c r="L35" s="2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="M35" s="2"/>
       <c r="N35" s="2"/>
@@ -2783,16 +2877,16 @@
       <c r="B36" s="15"/>
       <c r="C36" s="15"/>
       <c r="D36" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="G36" s="5" t="s">
         <v>147</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="G36" s="5" t="s">
-        <v>150</v>
       </c>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
@@ -2801,7 +2895,7 @@
         <v>6</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
@@ -2813,19 +2907,19 @@
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G37" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="H37" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="H37" s="1" t="s">
-        <v>156</v>
       </c>
       <c r="I37" s="1"/>
       <c r="J37" s="2"/>
@@ -2841,19 +2935,19 @@
       <c r="B38" s="16"/>
       <c r="C38" s="16"/>
       <c r="D38" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="G38" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="H38" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="H38" s="1" t="s">
-        <v>161</v>
       </c>
       <c r="I38" s="1"/>
       <c r="J38" s="2"/>
@@ -2869,16 +2963,16 @@
       <c r="B39" s="15"/>
       <c r="C39" s="15"/>
       <c r="D39" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="G39" s="5" t="s">
         <v>162</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="G39" s="5" t="s">
-        <v>165</v>
       </c>
       <c r="H39" s="5"/>
       <c r="I39" s="5"/>
@@ -2887,7 +2981,7 @@
         <v>6</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="M39" s="1"/>
       <c r="N39" s="1"/>
@@ -2896,19 +2990,19 @@
       <c r="A40" s="16"/>
       <c r="B40" s="16"/>
       <c r="C40" s="16" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="G40" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>169</v>
       </c>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
@@ -2925,19 +3019,19 @@
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
       <c r="D41" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G41" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="H41" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="H41" s="1" t="s">
-        <v>174</v>
       </c>
       <c r="I41" s="1"/>
       <c r="J41" s="2"/>
@@ -2953,16 +3047,16 @@
       <c r="B42" s="16"/>
       <c r="C42" s="16"/>
       <c r="D42" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="G42" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>178</v>
       </c>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
@@ -2979,16 +3073,16 @@
       <c r="B43" s="16"/>
       <c r="C43" s="16"/>
       <c r="D43" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G43" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>182</v>
       </c>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
@@ -3005,23 +3099,23 @@
       <c r="B44" s="16"/>
       <c r="C44" s="16"/>
       <c r="D44" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="G44" s="1" t="s">
         <v>183</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>186</v>
       </c>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
       <c r="J44" s="2"/>
       <c r="K44" s="16"/>
       <c r="L44" s="1" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
@@ -3033,16 +3127,16 @@
       <c r="B45" s="15"/>
       <c r="C45" s="15"/>
       <c r="D45" s="5" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="H45" s="5"/>
       <c r="I45" s="5"/>
@@ -3051,7 +3145,7 @@
         <v>6</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="M45" s="2"/>
       <c r="N45" s="2"/>
@@ -3063,16 +3157,16 @@
       <c r="B46" s="16"/>
       <c r="C46" s="16"/>
       <c r="D46" s="5" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
@@ -3081,7 +3175,7 @@
         <v>6</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="M46" s="1"/>
       <c r="N46" s="1"/>
@@ -3093,23 +3187,23 @@
       <c r="B47" s="16"/>
       <c r="C47" s="16"/>
       <c r="D47" s="1" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
       <c r="J47" s="2"/>
       <c r="K47" s="16"/>
       <c r="L47" s="2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="M47" s="2"/>
       <c r="N47" s="2"/>
@@ -3121,16 +3215,16 @@
       <c r="B48" s="16"/>
       <c r="C48" s="16"/>
       <c r="D48" s="1" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>217</v>
+        <v>301</v>
       </c>
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
@@ -3143,20 +3237,20 @@
     <row r="49" spans="1:14" ht="165" x14ac:dyDescent="0.25">
       <c r="A49" s="15"/>
       <c r="B49" s="15" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C49" s="15"/>
       <c r="D49" s="5" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="H49" s="5"/>
       <c r="I49" s="5"/>
@@ -3165,7 +3259,7 @@
         <v>6</v>
       </c>
       <c r="L49" s="1" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="M49" s="1"/>
       <c r="N49" s="1"/>
@@ -3177,16 +3271,16 @@
       <c r="B50" s="16"/>
       <c r="C50" s="16"/>
       <c r="D50" s="5" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="G50" s="5" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="H50" s="5"/>
       <c r="I50" s="5"/>
@@ -3195,7 +3289,7 @@
         <v>6</v>
       </c>
       <c r="L50" s="1" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="M50" s="1"/>
       <c r="N50" s="1"/>
@@ -3203,20 +3297,20 @@
     <row r="51" spans="1:14" ht="150" x14ac:dyDescent="0.25">
       <c r="A51" s="15"/>
       <c r="B51" s="15" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C51" s="15"/>
       <c r="D51" s="5" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="H51" s="5"/>
       <c r="I51" s="5"/>
@@ -3225,7 +3319,7 @@
         <v>6</v>
       </c>
       <c r="L51" s="1" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="M51" s="1"/>
       <c r="N51" s="1"/>
@@ -3233,20 +3327,20 @@
     <row r="52" spans="1:14" ht="150" x14ac:dyDescent="0.25">
       <c r="A52" s="16"/>
       <c r="B52" s="16" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C52" s="16"/>
       <c r="D52" s="5" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="H52" s="5"/>
       <c r="I52" s="5"/>
@@ -3255,269 +3349,267 @@
         <v>6</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
     </row>
-    <row r="53" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" ht="180" x14ac:dyDescent="0.25">
       <c r="A53" s="16"/>
       <c r="B53" s="16"/>
       <c r="C53" s="16"/>
       <c r="D53" s="1" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="H53" s="1"/>
+        <v>266</v>
+      </c>
+      <c r="H53" s="1" t="s">
+        <v>305</v>
+      </c>
       <c r="I53" s="1"/>
       <c r="J53" s="2"/>
       <c r="K53" s="16"/>
       <c r="L53" s="1" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="M53" s="1"/>
       <c r="N53" s="1"/>
     </row>
-    <row r="54" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" ht="225" x14ac:dyDescent="0.25">
       <c r="A54" s="16"/>
       <c r="B54" s="16"/>
       <c r="C54" s="16"/>
       <c r="D54" s="1" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>275</v>
+        <v>267</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>306</v>
       </c>
       <c r="I54" s="1"/>
       <c r="J54" s="2"/>
       <c r="K54" s="16"/>
       <c r="L54" s="1" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="M54" s="1"/>
       <c r="N54" s="1"/>
     </row>
-    <row r="55" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" ht="180" x14ac:dyDescent="0.25">
       <c r="A55" s="16"/>
       <c r="B55" s="16"/>
       <c r="C55" s="16"/>
       <c r="D55" s="1" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="H55" s="1"/>
+        <v>271</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>307</v>
+      </c>
       <c r="I55" s="1"/>
       <c r="J55" s="2"/>
       <c r="K55" s="16"/>
       <c r="L55" s="1" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="M55" s="1"/>
       <c r="N55" s="1"/>
     </row>
-    <row r="56" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" ht="225" x14ac:dyDescent="0.25">
       <c r="A56" s="16"/>
       <c r="B56" s="16"/>
       <c r="C56" s="16"/>
       <c r="D56" s="1" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="H56" s="1"/>
+        <v>272</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>308</v>
+      </c>
       <c r="I56" s="1"/>
       <c r="J56" s="2"/>
       <c r="K56" s="16"/>
       <c r="L56" s="1" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="M56" s="1"/>
       <c r="N56" s="1"/>
     </row>
-    <row r="57" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A57" s="16"/>
       <c r="B57" s="16"/>
       <c r="C57" s="16"/>
       <c r="D57" s="1" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="H57" s="1"/>
+        <v>273</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>309</v>
+      </c>
       <c r="I57" s="1"/>
       <c r="J57" s="2"/>
       <c r="K57" s="16"/>
       <c r="L57" s="1" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="M57" s="1"/>
       <c r="N57" s="1"/>
     </row>
-    <row r="58" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A58" s="16"/>
       <c r="B58" s="16"/>
       <c r="C58" s="16"/>
       <c r="D58" s="1" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>282</v>
+        <v>274</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>310</v>
       </c>
       <c r="I58" s="1"/>
       <c r="J58" s="2"/>
       <c r="K58" s="16"/>
       <c r="L58" s="1" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="M58" s="1"/>
       <c r="N58" s="1"/>
     </row>
-    <row r="59" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A59" s="16"/>
       <c r="B59" s="16"/>
       <c r="C59" s="16"/>
       <c r="D59" s="1" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>283</v>
+        <v>275</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>313</v>
       </c>
       <c r="I59" s="1"/>
       <c r="J59" s="2"/>
       <c r="K59" s="16"/>
       <c r="L59" s="1" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="M59" s="1"/>
       <c r="N59" s="1"/>
     </row>
-    <row r="60" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A60" s="16"/>
       <c r="B60" s="16"/>
       <c r="C60" s="16"/>
       <c r="D60" s="1" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>284</v>
+        <v>276</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>312</v>
       </c>
       <c r="I60" s="1"/>
       <c r="J60" s="2"/>
       <c r="K60" s="16"/>
       <c r="L60" s="1" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="M60" s="1"/>
       <c r="N60" s="1"/>
     </row>
-    <row r="61" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A61" s="16"/>
       <c r="B61" s="16"/>
       <c r="C61" s="16"/>
       <c r="D61" s="1" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>285</v>
+        <v>277</v>
+      </c>
+      <c r="H61" s="1" t="s">
+        <v>311</v>
       </c>
       <c r="I61" s="1"/>
       <c r="J61" s="2"/>
       <c r="K61" s="16"/>
       <c r="L61" s="1" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="M61" s="1"/>
       <c r="N61" s="1"/>
     </row>
-    <row r="62" spans="1:14" ht="90" x14ac:dyDescent="0.25">
-      <c r="A62" s="16"/>
-      <c r="B62" s="16"/>
-      <c r="C62" s="16"/>
-      <c r="D62" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="I62" s="1"/>
-      <c r="J62" s="2"/>
-      <c r="K62" s="16"/>
-      <c r="L62" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="M62" s="1"/>
-      <c r="N62" s="1"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N61" xr:uid="{B5C7E2F8-1D87-4E2E-8196-7F95EBE1FA6F}"/>
+  <autoFilter ref="A1:N60" xr:uid="{B5C7E2F8-1D87-4E2E-8196-7F95EBE1FA6F}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J62" xr:uid="{1C488EE4-4AD3-49DB-8EC8-8A5BD2F07EE9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J61" xr:uid="{1C488EE4-4AD3-49DB-8EC8-8A5BD2F07EE9}">
       <formula1>$W$1:$W$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Updated checklist with David Solins comments and minor updates to OVAL content
</commit_message>
<xml_diff>
--- a/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist_DRAFT.xlsx
+++ b/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist_DRAFT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flankspeed-my.sharepoint-mil.us/personal/jack_r_vanderpol_civ_us_navy_mil/Documents/Documents/github/SCAP-Self-Assertion/SCAP_1.4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="229" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C3F3B37-486F-443F-A6E1-64FE5EFB87ED}"/>
+  <xr:revisionPtr revIDLastSave="237" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74D108A6-EAC8-47D0-8CA8-374AC864099D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="90" windowWidth="29040" windowHeight="15510" xr2:uid="{91EDF8AA-12A4-463E-9EF6-D256E525D567}"/>
+    <workbookView xWindow="-120" yWindow="90" windowWidth="29040" windowHeight="15510" activeTab="2" xr2:uid="{91EDF8AA-12A4-463E-9EF6-D256E525D567}"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="2" r:id="rId1"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="322">
   <si>
     <t>The product’s documentation (printed or electronic) MUST assert that it uses SCAP and its component specifications and explain relevant details to the users of the product.</t>
   </si>
@@ -864,9 +864,6 @@
     <t xml:space="preserve">Not sure that CVSS is fully supported by SCAP, and I think current CVSS requires human interpretation based on the target?    </t>
   </si>
   <si>
-    <t>Either update and enforce or remove?</t>
-  </si>
-  <si>
     <t>SCAP.V.5000.1:  The vendor SHALL provide documentation listing all supported operating systems.</t>
   </si>
   <si>
@@ -946,9 +943,6 @@
   </si>
   <si>
     <t>NIWC Comments</t>
-  </si>
-  <si>
-    <t>&lt;Your Group&gt; Comments</t>
   </si>
   <si>
     <t>OVAL Board Consensus</t>
@@ -1184,9 +1178,6 @@
 1.  Review an Oracle or RHEL system and review rule results, confirming that any Gnome specific requirements are reported as not_applicable.</t>
   </si>
   <si>
-    <t>Recommend removing requirement.</t>
-  </si>
-  <si>
     <t>1.  Install all OVAL content from OVAL_Test_Content\agnostic.
 2.  Install all OVAL content from OVAL_Test_Content\windows.
 3.  Scan Windows targets with all OVAL content from steps 1-2, and review results.
@@ -1236,6 +1227,45 @@
     <t>1.  Install all OVAL content from OVAL_Test_Content\panos.
 2.  Scan panos targets with all OVAL content from step 1, and review results.
 All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t>Solin Comments</t>
+  </si>
+  <si>
+    <t>WDYM? How about it rejects something signed with an expired certificate, or a self-signed certificate from "The Hacker Collective" or something like that?</t>
+  </si>
+  <si>
+    <t>Why eliminate?</t>
+  </si>
+  <si>
+    <t>A note about the pointless carry-through requirements. Perhaps they can all be replaced by a single requirement, that the source datastream be contained in the result? Or something to that effect.  We don't want a side-effect of removing the requirement being that some joker always strips all the metadata away from the results.</t>
+  </si>
+  <si>
+    <t>No complaints here.</t>
+  </si>
+  <si>
+    <t>Agree</t>
+  </si>
+  <si>
+    <t>Maybe we should specify that products should not override anything that has been specified in the content itself.</t>
+  </si>
+  <si>
+    <t>Recommend removing requirement.
+It was mentioned in previous SCAP workgroups that this feature was not needed and may be removed from a future version of SCAP.    We can leave it in if the board thinks it has value.</t>
+  </si>
+  <si>
+    <t>This cepability is already tested by external variables from XCCDF, and this being  SCAP validation, I wasn't sure how much standalone OVAL features we needed to test.  
+Easy enough to add it back if it's of value.</t>
+  </si>
+  <si>
+    <t>Either update and enforce or remove?
+What we do with SCC is have a certicate store, and we verify that any digitally signed content can ba validated against that store, be it specific trusted public certs of the signer, or the CA Root cert that created the signers cert.
+This works for us, but i'm not sure if we want to force that on everyone else?  
+Ideally each tool should have some way to know how to trust content.   The challege of an expired certificate, is that you may end up rejecting content that is valid, and may not be updated again (Say old SCAP 1.3 validation content) due to the singers cert being expired?</t>
+  </si>
+  <si>
+    <t>This requirement seems pointless, the XML results will contain whatever CCE's are included in the content, and doesn't seem to add much value.
+Agree that a single requirement for all CVE/CCE/CPE data being passed through is likely wise.</t>
   </si>
 </sst>
 </file>
@@ -1734,12 +1764,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -1762,69 +1792,69 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B2" s="7"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B3" s="7"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B4" s="7"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B5" s="7"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B6" s="7"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B7" s="7"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B8" s="7"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B9" s="7"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B10" s="7"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B11" s="7"/>
     </row>
@@ -1853,7 +1883,8 @@
     <col min="9" max="9" width="22.42578125" style="3" customWidth="1"/>
     <col min="10" max="10" width="11.28515625" style="3" customWidth="1"/>
     <col min="11" max="11" width="13.140625" style="18" customWidth="1"/>
-    <col min="12" max="14" width="24.5703125" style="3" customWidth="1"/>
+    <col min="12" max="12" width="28.5703125" style="3" customWidth="1"/>
+    <col min="13" max="14" width="24.5703125" style="3" customWidth="1"/>
     <col min="15" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
@@ -1868,16 +1899,16 @@
         <v>5</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>21</v>
@@ -1892,16 +1923,16 @@
         <v>200</v>
       </c>
       <c r="L1" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="N1" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="M1" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>261</v>
-      </c>
       <c r="W1" s="13" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="105" x14ac:dyDescent="0.25">
@@ -1930,7 +1961,7 @@
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
       <c r="W2" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="210" x14ac:dyDescent="0.25">
@@ -1944,7 +1975,7 @@
         <v>65</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>66</v>
@@ -1954,12 +1985,12 @@
       <c r="J3" s="2"/>
       <c r="K3" s="14"/>
       <c r="L3" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="W3" s="3" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="135" x14ac:dyDescent="0.25">
@@ -2091,7 +2122,7 @@
         <v>32</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -2119,7 +2150,7 @@
         <v>35</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -2147,7 +2178,7 @@
         <v>38</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -2156,7 +2187,7 @@
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
     </row>
-    <row r="11" spans="1:23" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>6</v>
       </c>
@@ -2175,9 +2206,11 @@
       <c r="J11" s="2"/>
       <c r="K11" s="14"/>
       <c r="L11" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="M11" s="2"/>
+        <v>320</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>312</v>
+      </c>
       <c r="N11" s="2"/>
     </row>
     <row r="12" spans="1:23" ht="75" x14ac:dyDescent="0.25">
@@ -2199,7 +2232,7 @@
         <v>43</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -2229,7 +2262,7 @@
         <v>46</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
@@ -2287,7 +2320,7 @@
         <v>53</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
@@ -2313,7 +2346,7 @@
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -2373,7 +2406,7 @@
         <v>6</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
@@ -2430,8 +2463,12 @@
       <c r="K20" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
+      <c r="L20" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="M20" s="1" t="s">
+        <v>313</v>
+      </c>
       <c r="N20" s="5"/>
     </row>
     <row r="21" spans="1:14" ht="210" x14ac:dyDescent="0.25">
@@ -2459,9 +2496,11 @@
         <v>6</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="M21" s="2"/>
+        <v>318</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="N21" s="2"/>
     </row>
     <row r="22" spans="1:14" ht="180" x14ac:dyDescent="0.25">
@@ -2518,7 +2557,7 @@
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
     </row>
-    <row r="24" spans="1:14" s="17" customFormat="1" ht="165" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" s="17" customFormat="1" ht="210" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
         <v>6</v>
       </c>
@@ -2543,9 +2582,11 @@
         <v>6</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="M24" s="1"/>
+        <v>321</v>
+      </c>
+      <c r="M24" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="N24" s="1"/>
     </row>
     <row r="25" spans="1:14" ht="180" x14ac:dyDescent="0.25">
@@ -2721,7 +2762,9 @@
       <c r="L30" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="M30" s="2"/>
+      <c r="M30" s="2" t="s">
+        <v>315</v>
+      </c>
       <c r="N30" s="2"/>
     </row>
     <row r="31" spans="1:14" ht="150" x14ac:dyDescent="0.25">
@@ -2779,7 +2822,9 @@
       <c r="L32" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="M32" s="2"/>
+      <c r="M32" s="2" t="s">
+        <v>316</v>
+      </c>
       <c r="N32" s="2"/>
     </row>
     <row r="33" spans="1:14" ht="75" x14ac:dyDescent="0.25">
@@ -2801,7 +2846,7 @@
         <v>135</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="I33" s="1"/>
       <c r="J33" s="2"/>
@@ -3224,7 +3269,7 @@
         <v>212</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
@@ -3291,7 +3336,9 @@
       <c r="L50" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="M50" s="1"/>
+      <c r="M50" s="1" t="s">
+        <v>317</v>
+      </c>
       <c r="N50" s="1"/>
     </row>
     <row r="51" spans="1:14" ht="150" x14ac:dyDescent="0.25">
@@ -3359,25 +3406,25 @@
       <c r="B53" s="16"/>
       <c r="C53" s="16"/>
       <c r="D53" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="I53" s="1"/>
       <c r="J53" s="2"/>
       <c r="K53" s="16"/>
       <c r="L53" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="M53" s="1"/>
       <c r="N53" s="1"/>
@@ -3387,25 +3434,25 @@
       <c r="B54" s="16"/>
       <c r="C54" s="16"/>
       <c r="D54" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="I54" s="1"/>
       <c r="J54" s="2"/>
       <c r="K54" s="16"/>
       <c r="L54" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="M54" s="1"/>
       <c r="N54" s="1"/>
@@ -3415,25 +3462,25 @@
       <c r="B55" s="16"/>
       <c r="C55" s="16"/>
       <c r="D55" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="I55" s="1"/>
       <c r="J55" s="2"/>
       <c r="K55" s="16"/>
       <c r="L55" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="M55" s="1"/>
       <c r="N55" s="1"/>
@@ -3443,25 +3490,25 @@
       <c r="B56" s="16"/>
       <c r="C56" s="16"/>
       <c r="D56" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="I56" s="1"/>
       <c r="J56" s="2"/>
       <c r="K56" s="16"/>
       <c r="L56" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="M56" s="1"/>
       <c r="N56" s="1"/>
@@ -3471,25 +3518,25 @@
       <c r="B57" s="16"/>
       <c r="C57" s="16"/>
       <c r="D57" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="I57" s="1"/>
       <c r="J57" s="2"/>
       <c r="K57" s="16"/>
       <c r="L57" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="M57" s="1"/>
       <c r="N57" s="1"/>
@@ -3499,25 +3546,25 @@
       <c r="B58" s="16"/>
       <c r="C58" s="16"/>
       <c r="D58" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I58" s="1"/>
       <c r="J58" s="2"/>
       <c r="K58" s="16"/>
       <c r="L58" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="M58" s="1"/>
       <c r="N58" s="1"/>
@@ -3527,25 +3574,25 @@
       <c r="B59" s="16"/>
       <c r="C59" s="16"/>
       <c r="D59" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="I59" s="1"/>
       <c r="J59" s="2"/>
       <c r="K59" s="16"/>
       <c r="L59" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="M59" s="1"/>
       <c r="N59" s="1"/>
@@ -3555,25 +3602,25 @@
       <c r="B60" s="16"/>
       <c r="C60" s="16"/>
       <c r="D60" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="I60" s="1"/>
       <c r="J60" s="2"/>
       <c r="K60" s="16"/>
       <c r="L60" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="M60" s="1"/>
       <c r="N60" s="1"/>
@@ -3583,25 +3630,25 @@
       <c r="B61" s="16"/>
       <c r="C61" s="16"/>
       <c r="D61" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="I61" s="1"/>
       <c r="J61" s="2"/>
       <c r="K61" s="16"/>
       <c r="L61" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="M61" s="1"/>
       <c r="N61" s="1"/>

</xml_diff>

<commit_message>
Posting updates from 03/12/2026 board meeting
</commit_message>
<xml_diff>
--- a/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist_DRAFT.xlsx
+++ b/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist_DRAFT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flankspeed-my.sharepoint-mil.us/personal/jack_r_vanderpol_civ_us_navy_mil/Documents/Documents/github/SCAP-Self-Assertion/SCAP_1.4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="237" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74D108A6-EAC8-47D0-8CA8-374AC864099D}"/>
+  <xr:revisionPtr revIDLastSave="327" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{301EB302-3385-4CB7-B17E-4E1D60A27AEF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="90" windowWidth="29040" windowHeight="15510" activeTab="2" xr2:uid="{91EDF8AA-12A4-463E-9EF6-D256E525D567}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="SCAP 1.4 Self Assertion" sheetId="1" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SCAP 1.4 Self Assertion'!$A$1:$N$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SCAP 1.4 Self Assertion'!$A$1:$N$62</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'SCAP 1.4 Self Assertion'!$A:$J</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="341">
   <si>
     <t>The product’s documentation (printed or electronic) MUST assert that it uses SCAP and its component specifications and explain relevant details to the users of the product.</t>
   </si>
@@ -714,16 +714,10 @@
     <t>SCAP.V.3600.1: The vendor SHALL provide instructions on how product output can be generated that contains a listing of all security configuration issue items, with associated CCE IDs when available. Instructions SHALL include where the CCE IDs and the associated vendor supplied and/or official CCE descriptions can be located within the product output.</t>
   </si>
   <si>
-    <t>SCAP.T.3600.1: The tester SHALL visually inspect, within the product output, a non-vendor-directed set of 30 security configuration issue items, to ensure that the CCE IDs are displayed. This test is not intended to determine whether the product correctly maps to CCE or whether it provides a complete mapping.</t>
-  </si>
-  <si>
     <t>Wondering if this should be generalized to be xccdf:ident system data?  DISA uses CCI vs CCE</t>
   </si>
   <si>
     <t>Updated to state SCAP 1.3 vs SCAP 1.2, 1.1</t>
-  </si>
-  <si>
-    <t>Need to create testing notes for NIWC SCAP 1.4 content</t>
   </si>
   <si>
     <t>Since USGCB is no longer required, this test should be removed, unless we want to state that applications need to be compliant with all DISA STIGs?  Would take some research to know if that is possible or wise.</t>
@@ -949,10 +943,6 @@
   </si>
   <si>
     <t>If the product supports JunOS, it SHALL support all non-deprecated OVAL 5.12.2 tests AWS  schemas along with all core OVAL 5.12 features.</t>
-  </si>
-  <si>
-    <t>Updated SCAP 1.1 and 1.2 to be just SCAP 1.3.  Updated to require listing OVAL platforms and specific OVAL tests supported.  (much like the old MITRE OVAL adoption method)
-Need to determine if NIST will be able to publish information, or if it will be on some github page?</t>
   </si>
   <si>
     <t>If the product supports Linux, it SHALL support OVAL 5.12.2 tests for Independent, UNIX, Linux  schemas along with all core OVAL 5.12.2 features.</t>
@@ -1254,18 +1244,84 @@
 It was mentioned in previous SCAP workgroups that this feature was not needed and may be removed from a future version of SCAP.    We can leave it in if the board thinks it has value.</t>
   </si>
   <si>
-    <t>This cepability is already tested by external variables from XCCDF, and this being  SCAP validation, I wasn't sure how much standalone OVAL features we needed to test.  
-Easy enough to add it back if it's of value.</t>
-  </si>
-  <si>
-    <t>Either update and enforce or remove?
-What we do with SCC is have a certicate store, and we verify that any digitally signed content can ba validated against that store, be it specific trusted public certs of the signer, or the CA Root cert that created the signers cert.
-This works for us, but i'm not sure if we want to force that on everyone else?  
-Ideally each tool should have some way to know how to trust content.   The challege of an expired certificate, is that you may end up rejecting content that is valid, and may not be updated again (Say old SCAP 1.3 validation content) due to the singers cert being expired?</t>
-  </si>
-  <si>
     <t>This requirement seems pointless, the XML results will contain whatever CCE's are included in the content, and doesn't seem to add much value.
 Agree that a single requirement for all CVE/CCE/CPE data being passed through is likely wise.</t>
+  </si>
+  <si>
+    <t>SCAP.V.1000.1:The vendor SHALL provide documentation explaining how certificate verification occurs in their product.</t>
+  </si>
+  <si>
+    <t>SCAP.T.1000.1:   User the vendor product, the tester SHALL attempt to install and execute a SCAP source datastream that has been signed by a private/untrusted  digital cerificate.</t>
+  </si>
+  <si>
+    <t>Delete Requirement</t>
+  </si>
+  <si>
+    <t>Revert Requirement</t>
+  </si>
+  <si>
+    <t>More discussion needed</t>
+  </si>
+  <si>
+    <t>Delete if no content is available</t>
+  </si>
+  <si>
+    <t>SCAP.R.4900</t>
+  </si>
+  <si>
+    <t>SCAP.R.4901</t>
+  </si>
+  <si>
+    <t>The product shall include ident system information (CCE, CVE, CCI, etc ) from the XCCDF rule as part of the xccdf rule-result</t>
+  </si>
+  <si>
+    <t>SCAP.T.4500.1: The tester SHALL review the XCCDF rule results from any SCAP stream and confirm that the xccdf rule-result ident system information matches the corresponding xccdf rule ident system from the SCAP datastream.</t>
+  </si>
+  <si>
+    <t>The product shall include reference  ref_id, ref_url and source in OVAL results.  This could include CCE, CVE, CCI, etc..)</t>
+  </si>
+  <si>
+    <t>SCAP.V.4901.1: The vendor SHALL provide documentation (printed or electronic) indicating where oval reference information can be obtained</t>
+  </si>
+  <si>
+    <t>SCAP.V.4900.1: The vendor SHALL provide documentation (printed or electronic) indicating where xccdf ident system information can be obtained</t>
+  </si>
+  <si>
+    <t>SCAP.T.4500.1: The tester SHALL review the OVAL results from a the sample OVAL file and ensure that the results from the product contain the same reference information as the source OVAL XML document.</t>
+  </si>
+  <si>
+    <t>Delete Requirement, Replaced by R.4900 and R.4901</t>
+  </si>
+  <si>
+    <t>Created draft testing instructions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delete Requirement </t>
+  </si>
+  <si>
+    <t>SCA+D44:G44P.T.3600.1: The tester SHALL visually inspect, within the product output, a non-vendor-directed set of 30 security configuration issue items, to ensure that the CCE IDs are displayed. This test is not intended to determine whether the product correctly maps to CCE or whether it provides a complete mapping.</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>Updated SCAP 1.1 and 1.2 to be just SCAP 1.3.  Updated to require listing OVAL platforms and specific OVAL tests supported.  (much like the old MITRE OVAL adoption method)</t>
+  </si>
+  <si>
+    <t>1.  Install any of the content files in the R1100 directory.  They are old content files from NIST's SCAP 1.3 validation program, and are techically valid, but given the age, the certificate is expired, and the root cert that created it is likely not in any product's trusted certificate store.
+2.  Attempt to execute any of the files, and document the errors, likely that the certificate chain could not be verified.
+Note:  If the content does pass digitial signature validation, determine where the trusted certificate store is located, and remove the certificates that are used to verfy, and then retest.</t>
+  </si>
+  <si>
+    <t>1.  Install the oval_reference_text.xml content. 
+2.  Execute a scan using the product being tested.
+3.  Review all available reports, including OVAL XML and view resulting CVE, CCE, CCI references.</t>
+  </si>
+  <si>
+    <t>1.  Review a sample of XCCDF results from R700 and view XCCDF results to ensure that each rule-result contains an ident system, and the data in the rule-result matches the ident system from the content.</t>
+  </si>
+  <si>
+    <t>Review new test case</t>
   </si>
 </sst>
 </file>
@@ -1367,7 +1423,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1416,6 +1472,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1764,12 +1823,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -1792,69 +1851,69 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="B2" s="7"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B3" s="7"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="B4" s="7"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B5" s="7"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="B6" s="7"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="B7" s="7"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="B8" s="7"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="B9" s="7"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B10" s="7"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="B11" s="7"/>
     </row>
@@ -1866,10 +1925,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5C7E2F8-1D87-4E2E-8196-7F95EBE1FA6F}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:W61"/>
+  <dimension ref="A1:W63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" style="18" customWidth="1"/>
@@ -1899,16 +1958,16 @@
         <v>5</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>21</v>
@@ -1920,19 +1979,19 @@
         <v>9</v>
       </c>
       <c r="K1" s="12" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="W1" s="13" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="105" x14ac:dyDescent="0.25">
@@ -1961,7 +2020,7 @@
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
       <c r="W2" s="3" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="210" x14ac:dyDescent="0.25">
@@ -1975,7 +2034,7 @@
         <v>65</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>66</v>
@@ -1985,12 +2044,12 @@
       <c r="J3" s="2"/>
       <c r="K3" s="14"/>
       <c r="L3" s="2" t="s">
-        <v>261</v>
+        <v>336</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="W3" s="3" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="135" x14ac:dyDescent="0.25">
@@ -2122,7 +2181,7 @@
         <v>32</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -2150,7 +2209,7 @@
         <v>35</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -2178,7 +2237,7 @@
         <v>38</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -2187,7 +2246,7 @@
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
     </row>
-    <row r="11" spans="1:23" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" ht="255" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>6</v>
       </c>
@@ -2199,19 +2258,27 @@
       <c r="E11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
+      <c r="F11" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>337</v>
+      </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="14"/>
       <c r="L11" s="2" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="N11" s="2"/>
+        <v>309</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>340</v>
+      </c>
     </row>
     <row r="12" spans="1:23" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
@@ -2232,13 +2299,13 @@
         <v>43</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="14"/>
       <c r="L12" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
@@ -2262,14 +2329,12 @@
         <v>46</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="14"/>
-      <c r="L13" s="2" t="s">
-        <v>186</v>
-      </c>
+      <c r="L13" s="2"/>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
     </row>
@@ -2320,7 +2385,7 @@
         <v>53</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
@@ -2346,7 +2411,7 @@
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -2355,7 +2420,7 @@
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
     </row>
-    <row r="17" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>6</v>
       </c>
@@ -2380,12 +2445,14 @@
         <v>6</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-    </row>
-    <row r="18" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+      <c r="N17" s="2" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
         <v>6</v>
       </c>
@@ -2406,12 +2473,14 @@
         <v>6</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-    </row>
-    <row r="19" spans="1:14" s="17" customFormat="1" ht="150" x14ac:dyDescent="0.25">
+      <c r="N18" s="2" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" s="17" customFormat="1" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="15"/>
       <c r="B19" s="15"/>
       <c r="C19" s="14" t="s">
@@ -2437,7 +2506,9 @@
       </c>
       <c r="L19" s="5"/>
       <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
+      <c r="N19" s="2" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="20" spans="1:14" s="17" customFormat="1" ht="300" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
@@ -2445,31 +2516,29 @@
       </c>
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="F20" s="5" t="s">
+      <c r="F20" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="G20" s="5" t="s">
+      <c r="G20" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>319</v>
-      </c>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="1"/>
       <c r="M20" s="1" t="s">
-        <v>313</v>
-      </c>
-      <c r="N20" s="5"/>
+        <v>310</v>
+      </c>
+      <c r="N20" s="1" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="21" spans="1:14" ht="210" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
@@ -2493,15 +2562,17 @@
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
       <c r="K21" s="14" t="s">
-        <v>6</v>
+        <v>335</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="N21" s="2"/>
+        <v>310</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="22" spans="1:14" ht="180" x14ac:dyDescent="0.25">
       <c r="A22" s="14"/>
@@ -2557,7 +2628,7 @@
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
     </row>
-    <row r="24" spans="1:14" s="17" customFormat="1" ht="210" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" s="17" customFormat="1" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
         <v>6</v>
       </c>
@@ -2582,14 +2653,16 @@
         <v>6</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>314</v>
-      </c>
-      <c r="N24" s="1"/>
-    </row>
-    <row r="25" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+        <v>311</v>
+      </c>
+      <c r="N24" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
         <v>6</v>
       </c>
@@ -2614,12 +2687,14 @@
         <v>6</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="M25" s="1"/>
-      <c r="N25" s="1"/>
-    </row>
-    <row r="26" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+      <c r="N25" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
         <v>6</v>
       </c>
@@ -2644,10 +2719,12 @@
         <v>6</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="M26" s="1"/>
-      <c r="N26" s="1"/>
+      <c r="N26" s="2" t="s">
+        <v>331</v>
+      </c>
     </row>
     <row r="27" spans="1:14" ht="150" x14ac:dyDescent="0.25">
       <c r="A27" s="14"/>
@@ -2670,12 +2747,12 @@
       <c r="J27" s="2"/>
       <c r="K27" s="14"/>
       <c r="L27" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
     </row>
-    <row r="28" spans="1:14" ht="285" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="285" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="15"/>
       <c r="B28" s="15" t="s">
         <v>120</v>
@@ -2700,12 +2777,14 @@
         <v>6</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="M28" s="1"/>
-      <c r="N28" s="1"/>
-    </row>
-    <row r="29" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+      <c r="N28" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="15"/>
       <c r="B29" s="15" t="s">
         <v>120</v>
@@ -2730,12 +2809,14 @@
         <v>6</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="M29" s="1"/>
-      <c r="N29" s="1"/>
-    </row>
-    <row r="30" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+      <c r="N29" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
         <v>6</v>
       </c>
@@ -2760,12 +2841,14 @@
         <v>6</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="N30" s="2"/>
+        <v>312</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>333</v>
+      </c>
     </row>
     <row r="31" spans="1:14" ht="150" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
@@ -2790,12 +2873,12 @@
       <c r="J31" s="2"/>
       <c r="K31" s="16"/>
       <c r="L31" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
     </row>
-    <row r="32" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
         <v>6</v>
       </c>
@@ -2820,12 +2903,14 @@
         <v>6</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="N32" s="2"/>
+        <v>313</v>
+      </c>
+      <c r="N32" s="2" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="33" spans="1:14" ht="75" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
@@ -2846,13 +2931,13 @@
         <v>135</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="I33" s="1"/>
       <c r="J33" s="2"/>
       <c r="K33" s="16"/>
       <c r="L33" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
@@ -2882,7 +2967,7 @@
       <c r="J34" s="2"/>
       <c r="K34" s="16"/>
       <c r="L34" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
@@ -2910,12 +2995,12 @@
       <c r="J35" s="2"/>
       <c r="K35" s="16"/>
       <c r="L35" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="M35" s="2"/>
       <c r="N35" s="2"/>
     </row>
-    <row r="36" spans="1:14" ht="255" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="255" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
         <v>6</v>
       </c>
@@ -2940,10 +3025,12 @@
         <v>6</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="M36" s="2"/>
-      <c r="N36" s="2"/>
+      <c r="N36" s="2" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="37" spans="1:14" ht="390" x14ac:dyDescent="0.25">
       <c r="A37" s="16" t="s">
@@ -3001,7 +3088,7 @@
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
     </row>
-    <row r="39" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
         <v>6</v>
       </c>
@@ -3026,10 +3113,12 @@
         <v>6</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="M39" s="1"/>
-      <c r="N39" s="1"/>
+      <c r="N39" s="2" t="s">
+        <v>331</v>
+      </c>
     </row>
     <row r="40" spans="1:14" ht="90" x14ac:dyDescent="0.25">
       <c r="A40" s="16"/>
@@ -3137,51 +3226,55 @@
       <c r="M43" s="2"/>
       <c r="N43" s="2"/>
     </row>
-    <row r="44" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B44" s="16"/>
       <c r="C44" s="16"/>
-      <c r="D44" s="1" t="s">
+      <c r="D44" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="E44" s="1" t="s">
+      <c r="E44" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="F44" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="G44" s="1" t="s">
-        <v>183</v>
+      <c r="G44" s="5" t="s">
+        <v>334</v>
       </c>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
       <c r="J44" s="2"/>
-      <c r="K44" s="16"/>
+      <c r="K44" s="16" t="s">
+        <v>6</v>
+      </c>
       <c r="L44" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="M44" s="1"/>
-      <c r="N44" s="1"/>
-    </row>
-    <row r="45" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+      <c r="N44" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B45" s="15"/>
       <c r="C45" s="15"/>
       <c r="D45" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="F45" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="E45" s="5" t="s">
+      <c r="G45" s="5" t="s">
         <v>196</v>
-      </c>
-      <c r="F45" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="G45" s="5" t="s">
-        <v>198</v>
       </c>
       <c r="H45" s="5"/>
       <c r="I45" s="5"/>
@@ -3190,28 +3283,30 @@
         <v>6</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="M45" s="2"/>
-      <c r="N45" s="2"/>
-    </row>
-    <row r="46" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+      <c r="N45" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B46" s="16"/>
       <c r="C46" s="16"/>
       <c r="D46" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="F46" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="E46" s="5" t="s">
+      <c r="G46" s="5" t="s">
         <v>202</v>
-      </c>
-      <c r="F46" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="G46" s="5" t="s">
-        <v>204</v>
       </c>
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
@@ -3220,10 +3315,12 @@
         <v>6</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="M46" s="1"/>
-      <c r="N46" s="1"/>
+      <c r="N46" s="2" t="s">
+        <v>331</v>
+      </c>
     </row>
     <row r="47" spans="1:14" ht="135" x14ac:dyDescent="0.25">
       <c r="A47" s="16" t="s">
@@ -3232,23 +3329,23 @@
       <c r="B47" s="16"/>
       <c r="C47" s="16"/>
       <c r="D47" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="F47" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="E47" s="1" t="s">
+      <c r="G47" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="G47" s="1" t="s">
-        <v>209</v>
       </c>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
       <c r="J47" s="2"/>
       <c r="K47" s="16"/>
       <c r="L47" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="M47" s="2"/>
       <c r="N47" s="2"/>
@@ -3260,16 +3357,16 @@
       <c r="B48" s="16"/>
       <c r="C48" s="16"/>
       <c r="D48" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F48" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="E48" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="F48" s="1" t="s">
-        <v>212</v>
-      </c>
       <c r="G48" s="1" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
@@ -3279,23 +3376,23 @@
       <c r="M48" s="1"/>
       <c r="N48" s="1"/>
     </row>
-    <row r="49" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="15"/>
       <c r="B49" s="15" t="s">
         <v>120</v>
       </c>
       <c r="C49" s="15"/>
       <c r="D49" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="F49" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="E49" s="5" t="s">
+      <c r="G49" s="5" t="s">
         <v>214</v>
-      </c>
-      <c r="F49" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="G49" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="H49" s="5"/>
       <c r="I49" s="5"/>
@@ -3304,28 +3401,30 @@
         <v>6</v>
       </c>
       <c r="L49" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="M49" s="1"/>
-      <c r="N49" s="1"/>
-    </row>
-    <row r="50" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+      <c r="N49" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B50" s="16"/>
       <c r="C50" s="16"/>
       <c r="D50" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="F50" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="E50" s="5" t="s">
+      <c r="G50" s="5" t="s">
         <v>219</v>
-      </c>
-      <c r="F50" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="G50" s="5" t="s">
-        <v>221</v>
       </c>
       <c r="H50" s="5"/>
       <c r="I50" s="5"/>
@@ -3334,30 +3433,32 @@
         <v>6</v>
       </c>
       <c r="L50" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="M50" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="N50" s="1"/>
-    </row>
-    <row r="51" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+        <v>314</v>
+      </c>
+      <c r="N50" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="15"/>
       <c r="B51" s="15" t="s">
         <v>120</v>
       </c>
       <c r="C51" s="15"/>
       <c r="D51" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="F51" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="E51" s="5" t="s">
+      <c r="G51" s="5" t="s">
         <v>224</v>
-      </c>
-      <c r="F51" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="G51" s="5" t="s">
-        <v>226</v>
       </c>
       <c r="H51" s="5"/>
       <c r="I51" s="5"/>
@@ -3366,28 +3467,30 @@
         <v>6</v>
       </c>
       <c r="L51" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="M51" s="1"/>
-      <c r="N51" s="1"/>
-    </row>
-    <row r="52" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+      <c r="N51" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="16"/>
       <c r="B52" s="16" t="s">
         <v>120</v>
       </c>
       <c r="C52" s="16"/>
       <c r="D52" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="F52" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="E52" s="5" t="s">
+      <c r="G52" s="5" t="s">
         <v>228</v>
-      </c>
-      <c r="F52" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="G52" s="5" t="s">
-        <v>230</v>
       </c>
       <c r="H52" s="5"/>
       <c r="I52" s="5"/>
@@ -3396,91 +3499,93 @@
         <v>6</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="M52" s="1"/>
-      <c r="N52" s="1"/>
-    </row>
-    <row r="53" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+      <c r="N52" s="2" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" s="19" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A53" s="16"/>
       <c r="B53" s="16"/>
       <c r="C53" s="16"/>
       <c r="D53" s="1" t="s">
-        <v>233</v>
+        <v>323</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>252</v>
+        <v>325</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>232</v>
+        <v>329</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>264</v>
+        <v>326</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>302</v>
+        <v>339</v>
       </c>
       <c r="I53" s="1"/>
-      <c r="J53" s="2"/>
+      <c r="J53" s="1"/>
       <c r="K53" s="16"/>
-      <c r="L53" s="1" t="s">
-        <v>234</v>
-      </c>
+      <c r="L53" s="1"/>
       <c r="M53" s="1"/>
-      <c r="N53" s="1"/>
-    </row>
-    <row r="54" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+      <c r="N53" s="1" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" s="19" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A54" s="16"/>
       <c r="B54" s="16"/>
       <c r="C54" s="16"/>
       <c r="D54" s="1" t="s">
-        <v>235</v>
+        <v>324</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>262</v>
+        <v>327</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>242</v>
+        <v>328</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>265</v>
+        <v>330</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>303</v>
+        <v>338</v>
       </c>
       <c r="I54" s="1"/>
-      <c r="J54" s="2"/>
+      <c r="J54" s="1"/>
       <c r="K54" s="16"/>
-      <c r="L54" s="1" t="s">
-        <v>234</v>
-      </c>
+      <c r="L54" s="1"/>
       <c r="M54" s="1"/>
-      <c r="N54" s="1"/>
+      <c r="N54" s="1" t="s">
+        <v>340</v>
+      </c>
     </row>
     <row r="55" spans="1:14" ht="180" x14ac:dyDescent="0.25">
       <c r="A55" s="16"/>
       <c r="B55" s="16"/>
       <c r="C55" s="16"/>
       <c r="D55" s="1" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>243</v>
+        <v>230</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="I55" s="1"/>
       <c r="J55" s="2"/>
       <c r="K55" s="16"/>
       <c r="L55" s="1" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="M55" s="1"/>
       <c r="N55" s="1"/>
@@ -3490,81 +3595,81 @@
       <c r="B56" s="16"/>
       <c r="C56" s="16"/>
       <c r="D56" s="1" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="I56" s="1"/>
       <c r="J56" s="2"/>
       <c r="K56" s="16"/>
       <c r="L56" s="1" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="M56" s="1"/>
       <c r="N56" s="1"/>
     </row>
-    <row r="57" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" ht="180" x14ac:dyDescent="0.25">
       <c r="A57" s="16"/>
       <c r="B57" s="16"/>
       <c r="C57" s="16"/>
       <c r="D57" s="1" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="I57" s="1"/>
       <c r="J57" s="2"/>
       <c r="K57" s="16"/>
       <c r="L57" s="1" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="M57" s="1"/>
       <c r="N57" s="1"/>
     </row>
-    <row r="58" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" ht="225" x14ac:dyDescent="0.25">
       <c r="A58" s="16"/>
       <c r="B58" s="16"/>
       <c r="C58" s="16"/>
       <c r="D58" s="1" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I58" s="1"/>
       <c r="J58" s="2"/>
       <c r="K58" s="16"/>
       <c r="L58" s="1" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="M58" s="1"/>
       <c r="N58" s="1"/>
@@ -3574,25 +3679,25 @@
       <c r="B59" s="16"/>
       <c r="C59" s="16"/>
       <c r="D59" s="1" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="I59" s="1"/>
       <c r="J59" s="2"/>
       <c r="K59" s="16"/>
       <c r="L59" s="1" t="s">
-        <v>251</v>
+        <v>232</v>
       </c>
       <c r="M59" s="1"/>
       <c r="N59" s="1"/>
@@ -3602,25 +3707,25 @@
       <c r="B60" s="16"/>
       <c r="C60" s="16"/>
       <c r="D60" s="1" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="I60" s="1"/>
       <c r="J60" s="2"/>
       <c r="K60" s="16"/>
       <c r="L60" s="1" t="s">
-        <v>251</v>
+        <v>232</v>
       </c>
       <c r="M60" s="1"/>
       <c r="N60" s="1"/>
@@ -3630,33 +3735,98 @@
       <c r="B61" s="16"/>
       <c r="C61" s="16"/>
       <c r="D61" s="1" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="I61" s="1"/>
       <c r="J61" s="2"/>
       <c r="K61" s="16"/>
       <c r="L61" s="1" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="M61" s="1"/>
       <c r="N61" s="1"/>
     </row>
+    <row r="62" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+      <c r="A62" s="16"/>
+      <c r="B62" s="16"/>
+      <c r="C62" s="16"/>
+      <c r="D62" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="H62" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="I62" s="1"/>
+      <c r="J62" s="2"/>
+      <c r="K62" s="16" t="s">
+        <v>335</v>
+      </c>
+      <c r="L62" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="N62" s="1" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+      <c r="A63" s="16"/>
+      <c r="B63" s="16"/>
+      <c r="C63" s="16"/>
+      <c r="D63" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="I63" s="1"/>
+      <c r="J63" s="2"/>
+      <c r="K63" s="16"/>
+      <c r="L63" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="M63" s="1"/>
+      <c r="N63" s="1"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N60" xr:uid="{B5C7E2F8-1D87-4E2E-8196-7F95EBE1FA6F}"/>
+  <autoFilter ref="A1:N62" xr:uid="{B5C7E2F8-1D87-4E2E-8196-7F95EBE1FA6F}">
+    <filterColumn colId="10">
+      <filters blank="1">
+        <filter val="TBD"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J61" xr:uid="{1C488EE4-4AD3-49DB-8EC8-8A5BD2F07EE9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J63" xr:uid="{1C488EE4-4AD3-49DB-8EC8-8A5BD2F07EE9}">
       <formula1>$W$1:$W$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fixed typo in new testcase
</commit_message>
<xml_diff>
--- a/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist_DRAFT.xlsx
+++ b/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist_DRAFT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flankspeed-my.sharepoint-mil.us/personal/jack_r_vanderpol_civ_us_navy_mil/Documents/Documents/github/SCAP-Self-Assertion/SCAP_1.4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="327" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{301EB302-3385-4CB7-B17E-4E1D60A27AEF}"/>
+  <xr:revisionPtr revIDLastSave="335" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2AC1B8AF-91EE-4FCE-85C3-C36C32B84788}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="90" windowWidth="29040" windowHeight="15510" activeTab="2" xr2:uid="{91EDF8AA-12A4-463E-9EF6-D256E525D567}"/>
+    <workbookView xWindow="-120" yWindow="90" windowWidth="29040" windowHeight="15510" xr2:uid="{91EDF8AA-12A4-463E-9EF6-D256E525D567}"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="2" r:id="rId1"/>
@@ -1308,11 +1308,6 @@
     <t>Updated SCAP 1.1 and 1.2 to be just SCAP 1.3.  Updated to require listing OVAL platforms and specific OVAL tests supported.  (much like the old MITRE OVAL adoption method)</t>
   </si>
   <si>
-    <t>1.  Install any of the content files in the R1100 directory.  They are old content files from NIST's SCAP 1.3 validation program, and are techically valid, but given the age, the certificate is expired, and the root cert that created it is likely not in any product's trusted certificate store.
-2.  Attempt to execute any of the files, and document the errors, likely that the certificate chain could not be verified.
-Note:  If the content does pass digitial signature validation, determine where the trusted certificate store is located, and remove the certificates that are used to verfy, and then retest.</t>
-  </si>
-  <si>
     <t>1.  Install the oval_reference_text.xml content. 
 2.  Execute a scan using the product being tested.
 3.  Review all available reports, including OVAL XML and view resulting CVE, CCE, CCI references.</t>
@@ -1322,6 +1317,11 @@
   </si>
   <si>
     <t>Review new test case</t>
+  </si>
+  <si>
+    <t>1.  Install any of the content files in the R1000 directory.  They are old content files from NIST's SCAP 1.3 validation program, and are techically valid, but given the age, the certificate is expired, and the root cert that created it is likely not in any product's trusted certificate store.
+2.  Attempt to execute any of the files, and document the errors, likely that the certificate chain could not be verified.
+Note:  If the content does pass digitial signature validation, determine where the trusted certificate store is located, and remove the certificates that are used to verfy, and then retest.</t>
   </si>
 </sst>
 </file>
@@ -2265,7 +2265,7 @@
         <v>318</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -2277,7 +2277,7 @@
         <v>309</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="12" spans="1:23" ht="75" x14ac:dyDescent="0.25">
@@ -3523,7 +3523,7 @@
         <v>326</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="I53" s="1"/>
       <c r="J53" s="1"/>
@@ -3531,7 +3531,7 @@
       <c r="L53" s="1"/>
       <c r="M53" s="1"/>
       <c r="N53" s="1" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="54" spans="1:14" s="19" customFormat="1" ht="105" x14ac:dyDescent="0.25">
@@ -3551,7 +3551,7 @@
         <v>330</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="I54" s="1"/>
       <c r="J54" s="1"/>
@@ -3559,7 +3559,7 @@
       <c r="L54" s="1"/>
       <c r="M54" s="1"/>
       <c r="N54" s="1" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="55" spans="1:14" ht="180" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated test instructions for R1900, replacing NIST content with OVAL test content implementation
</commit_message>
<xml_diff>
--- a/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist_DRAFT.xlsx
+++ b/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist_DRAFT.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flankspeed-my.sharepoint-mil.us/personal/jack_r_vanderpol_civ_us_navy_mil/Documents/Documents/github/SCAP-Self-Assertion/SCAP_1.4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="335" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2AC1B8AF-91EE-4FCE-85C3-C36C32B84788}"/>
+  <xr:revisionPtr revIDLastSave="339" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D8EE275-7424-4C12-ACFF-67B536DF1815}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="90" windowWidth="29040" windowHeight="15510" xr2:uid="{91EDF8AA-12A4-463E-9EF6-D256E525D567}"/>
   </bookViews>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="342">
   <si>
     <t>The product’s documentation (printed or electronic) MUST assert that it uses SCAP and its component specifications and explain relevant details to the users of the product.</t>
   </si>
@@ -1322,6 +1322,11 @@
     <t>1.  Install any of the content files in the R1000 directory.  They are old content files from NIST's SCAP 1.3 validation program, and are techically valid, but given the age, the certificate is expired, and the root cert that created it is likely not in any product's trusted certificate store.
 2.  Attempt to execute any of the files, and document the errors, likely that the certificate chain could not be verified.
 Note:  If the content does pass digitial signature validation, determine where the trusted certificate store is located, and remove the certificates that are used to verfy, and then retest.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.  Install oval-def-ext.zip from the R1900 directory.    This should install both the OVAL content file and the OVAL Variables XML file into the product.   If after performing a scan, the product cannot locate the OVAL Variables file, refer to product documentation on how to install external variables XML files.
+2.  Scan any target with the oval-def-ext content enabled, oval defintion and all tests should return true if the product supports external variables.
+</t>
   </si>
 </sst>
 </file>
@@ -2528,7 +2533,9 @@
       <c r="G20" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="H20" s="1"/>
+      <c r="H20" s="1" t="s">
+        <v>341</v>
+      </c>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="16"/>

</xml_diff>